<commit_message>
generate insulin dosage data
</commit_message>
<xml_diff>
--- a/excel/t1d_metric_dictionary_and_qa.xlsx
+++ b/excel/t1d_metric_dictionary_and_qa.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -20,6 +20,7 @@
     <sheet name="Dashboard_Mockup" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -112,7 +113,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,49 +160,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="17">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -233,34 +192,46 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -276,21 +247,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F95507B-16A5-42DE-B9DF-9850896A825C}" name="qa_checks_table" displayName="qa_checks_table" ref="A1:L21" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F95507B-16A5-42DE-B9DF-9850896A825C}" name="qa_checks_table" displayName="qa_checks_table" ref="A1:L21" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A1:L21" xr:uid="{9F95507B-16A5-42DE-B9DF-9850896A825C}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{2AE4DD3F-0726-4C8B-A19C-2483596DEC4D}" name="check_id" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{15558B60-12B0-45D8-8F81-8B5B51AB6788}" name="check_category" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{7C12F6A4-92DA-4544-8EB9-3DBB84E0447A}" name="check_name" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{33C5B67F-B2F1-476D-9AE8-8FF68FA66492}" name="check_description" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{EBEB94E5-B99A-481C-BCFA-45032DDFE45E}" name="source_layer" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{62BE9463-9F43-4928-A97D-C011BFE2AA86}" name="source_table_or_file" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{4DB7230A-2FE3-4AF3-845C-F0C6C9051053}" name="expected_result" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{E2DF9C55-FAF5-41B5-9D83-22C305E42199}" name="actual_result" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{F2D62DEE-E737-4103-A69B-6F4B9E9D8220}" name="status" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{D3F07466-4636-4A4E-A055-5B6540B40E1F}" name="checked_by" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{2B0A0704-CDE7-4266-AFD2-2175EBFF4B12}" name="check_date" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{563B16EB-5ECC-43A5-9B7D-673AC47AA45F}" name="notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{2AE4DD3F-0726-4C8B-A19C-2483596DEC4D}" name="check_id" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{15558B60-12B0-45D8-8F81-8B5B51AB6788}" name="check_category" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{7C12F6A4-92DA-4544-8EB9-3DBB84E0447A}" name="check_name" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{33C5B67F-B2F1-476D-9AE8-8FF68FA66492}" name="check_description" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{EBEB94E5-B99A-481C-BCFA-45032DDFE45E}" name="source_layer" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{62BE9463-9F43-4928-A97D-C011BFE2AA86}" name="source_table_or_file" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{4DB7230A-2FE3-4AF3-845C-F0C6C9051053}" name="expected_result" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{E2DF9C55-FAF5-41B5-9D83-22C305E42199}" name="actual_result" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{F2D62DEE-E737-4103-A69B-6F4B9E9D8220}" name="status" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{D3F07466-4636-4A4E-A055-5B6540B40E1F}" name="checked_by" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{2B0A0704-CDE7-4266-AFD2-2175EBFF4B12}" name="check_date" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{563B16EB-5ECC-43A5-9B7D-673AC47AA45F}" name="notes" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -614,7 +585,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF9A7223-EBEA-459A-BE39-C508BAA038D0}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -623,7 +594,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0934BE5-7B9D-43F5-A9E2-CAA57E265E59}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -632,23 +603,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333A6998-C701-4ED3-A735-613ED5815808}">
   <dimension ref="A1:M21"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.296875" customWidth="1"/>
-    <col min="2" max="2" width="14.19921875" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14.21875" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="16.3984375" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="17.5" customWidth="1"/>
-    <col min="7" max="7" width="14.59765625" customWidth="1"/>
-    <col min="8" max="8" width="12.296875" customWidth="1"/>
-    <col min="10" max="10" width="11.5" customWidth="1"/>
-    <col min="11" max="11" width="12.3984375" customWidth="1"/>
-    <col min="12" max="12" width="11.19921875" customWidth="1"/>
-    <col min="13" max="13" width="8.796875" style="1"/>
+    <col min="6" max="6" width="17.44140625" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" customWidth="1"/>
+    <col min="11" max="11" width="12.44140625" customWidth="1"/>
+    <col min="12" max="12" width="11.21875" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -686,7 +657,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -724,7 +695,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -738,7 +709,7 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -752,7 +723,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -766,7 +737,7 @@
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -780,7 +751,7 @@
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -794,7 +765,7 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -808,7 +779,7 @@
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -822,7 +793,7 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -836,7 +807,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -850,7 +821,7 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -864,7 +835,7 @@
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -878,7 +849,7 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -892,7 +863,7 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -906,7 +877,7 @@
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -920,7 +891,7 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -934,7 +905,7 @@
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -948,7 +919,7 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -962,7 +933,7 @@
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -976,7 +947,7 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -992,14 +963,14 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="I2:I200">
-    <cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",I2)))</formula>
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Review">
+      <formula>NOT(ISERROR(SEARCH("Review",I2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="2" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",I2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="1" operator="containsText" text="Review">
-      <formula>NOT(ISERROR(SEARCH("Review",I2)))</formula>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -1018,7 +989,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72CAB481-3C03-4332-AE95-35D85DA26E83}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1027,7 +998,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7486A5E4-215E-4496-B2A6-E3B845E3383D}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
create patient summary view
</commit_message>
<xml_diff>
--- a/excel/t1d_metric_dictionary_and_qa.xlsx
+++ b/excel/t1d_metric_dictionary_and_qa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joshua\Documents\type1-diabetes-analytics\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DEDB022-4FF5-4B30-AED1-BFFEDB9B63B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C5CD0B-7EBC-426F-B265-B2F30D8D3D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{7DA93E7F-9955-4DAF-962B-AE3274BCE9C0}"/>
   </bookViews>
@@ -605,17 +605,18 @@
   <dimension ref="A1:M21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" customWidth="1"/>
-    <col min="2" max="2" width="14.21875" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" customWidth="1"/>
-    <col min="11" max="11" width="12.44140625" customWidth="1"/>
-    <col min="12" max="12" width="11.21875" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1"/>
   </cols>
   <sheetData>

</xml_diff>